<commit_message>
docs/unlocks_and_tutorials.xlsx: the win streak starts November 4 (level 7 on).
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/unlocks_and_tutorials.xlsx
+++ b/docs/unlocks_and_tutorials.xlsx
@@ -7,7 +7,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By level'!$A$1:$F$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dates and recurring'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dates and recurring'!$A$1:$F$13</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -417,7 +417,7 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 7</t>
+          <t xml:space="preserve">Level 7 (from Nov 4)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
@@ -432,7 +432,7 @@
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Shown as it happens: the flame counter under the hearts, a banner when free rocks fly, a line on the win card.</t>
+          <t xml:space="preserve">Off until Nov 4, 2026, then shown as it happens: the flame counter under the hearts, a banner when free rocks fly, a line on the win card.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
@@ -1361,7 +1361,7 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nov 11, 2026</t>
+          <t xml:space="preserve">Nov 4, 2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
@@ -1371,186 +1371,218 @@
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Leaderboards (Ranks) open</t>
+          <t xml:space="preserve">Win streak starts</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tab tagged NOV 11 until then: "Leaderboards open November 11!"</t>
+          <t xml:space="preserve">No announcement: the flame counter appears under the hearts after a win from level 7 on</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Ranks tab</t>
+          <t xml:space="preserve">Game / Home</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Daily, weekly and season boards; the first season board counts from today to Dec 1 (20 days)</t>
+          <t xml:space="preserve">Before Nov 4 no level counts toward a streak</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nov 26-29, 2026</t>
+          <t xml:space="preserve">Nov 11, 2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Sale</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Hatch Day Feast (level 7+)</t>
+          <t xml:space="preserve">Leaderboards (Ranks) open</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Pop-up on Home</t>
+          <t xml:space="preserve">Tab tagged NOV 11 until then: "Leaderboards open November 11!"</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Ranks tab</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Once</t>
+          <t xml:space="preserve">Daily, weekly and season boards; the first season board counts from today to Dec 1 (20 days)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dec 1, 2026</t>
+          <t xml:space="preserve">Nov 26-29, 2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Season</t>
+          <t xml:space="preserve">Sale</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Battle Pass season 2 (Christmas) + voyage to a new planet; season leaderboard resets</t>
+          <t xml:space="preserve">Hatch Day Feast (level 7+)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The voyage plays on the next Home visit</t>
+          <t xml:space="preserve">Pop-up on Home</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Battle Pass / Home</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Seasons are 28 days from here</t>
+          <t xml:space="preserve">Once</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dec 9, 2026</t>
+          <t xml:space="preserve">Dec 1, 2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Feature</t>
+          <t xml:space="preserve">Season</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Teams (Clubs) open</t>
+          <t xml:space="preserve">Battle Pass season 2 (Christmas) + voyage to a new planet; season leaderboard resets</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tab tagged DEC 9 until then: "Teams open December 9!"</t>
+          <t xml:space="preserve">The voyage plays on the next Home visit</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Clubs tab</t>
+          <t xml:space="preserve">Battle Pass / Home</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Also needs level 25</t>
+          <t xml:space="preserve">Seasons are 28 days from here</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Dec 29, 2026</t>
+          <t xml:space="preserve">Dec 9, 2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Season</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Season 3 (New Year's)</t>
+          <t xml:space="preserve">Teams (Clubs) open</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Voyage</t>
+          <t xml:space="preserve">Tab tagged DEC 9 until then: "Teams open December 9!"</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Battle Pass / Home</t>
+          <t xml:space="preserve">Clubs tab</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Also needs level 25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Dec 29, 2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Season</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Season 3 (New Year's)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Voyage</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Battle Pass / Home</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Jan 26, 2027</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr" s="0">
+      <c r="B13" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Season</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="0">
+      <c r="C13" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Season 4 (Valentine's)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="0">
+      <c r="D13" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Voyage</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="0">
+      <c r="E13" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Battle Pass / Home</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr" s="0">
+      <c r="F13" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Then the four themes repeat</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
The piece counter's card waits its turn: last in the lesson queue, so it shows on the first level from 2 on with no other lesson (level 5 for a new player) and never pushes the bomb, Any Piece or blocker lessons back a level. The 1.2 release notes and docs/unlocks_and_tutorials.xlsx cover the counter.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/unlocks_and_tutorials.xlsx
+++ b/docs/unlocks_and_tutorials.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Dates and recurring" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By level'!$A$1:$F$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By level'!$A$1:$F$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dates and recurring'!$A$1:$F$13</definedName>
   </definedNames>
 </workbook>
@@ -321,7 +321,7 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 5</t>
+          <t xml:space="preserve">Level 1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
@@ -331,22 +331,22 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Collection tab</t>
+          <t xml:space="preserve">Piece counter</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Walkthrough after winning level 4: what the Collection is, a coin gift, tap Doc, tap Buy, Doc is yours; Collection levels add +1% materials.</t>
+          <t xml:space="preserve">The pill under the tray counts down from the level's budget (no card yet)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Collection</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Doc is the first critter adopted</t>
+          <t xml:space="preserve">Each level's own budget (levels/piece_budgets.json), 10-31 pieces. Out of pieces: a heart buys one random piece; a continue or heart ad adds 5. Not on challenges</t>
         </is>
       </c>
     </row>
@@ -358,34 +358,34 @@
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Feature</t>
+          <t xml:space="preserve">Tutorial</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Camp building + the mine</t>
+          <t xml:space="preserve">Piece counter card</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Camp callout on the first Home visit with build spots: the world glides to the campfire; tap a plus to build. Camp Lv 5 opens the ship.</t>
+          <t xml:space="preserve">1 card on the counter: run out and each extra piece costs a heart, at random</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The mine under the ship fills with materials over time</t>
+          <t xml:space="preserve">The first level from 2 on with no other lesson (or the first time the pieces run out)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 7</t>
+          <t xml:space="preserve">Level 5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
@@ -395,29 +395,29 @@
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Chest tray, Battle Pass, 7-Day Eggsperience</t>
+          <t xml:space="preserve">Collection tab</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home walkthrough: a free Common chest to unlock (gated taps), wins earn chests (3 wins each), the Battle Pass (hearts left become stars), the Eggsperience quests.</t>
+          <t xml:space="preserve">Walkthrough after winning level 4: what the Collection is, a coin gift, tap Doc, tap Buy, Doc is yours; Collection levels add +1% materials.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Collection</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Stars, daily and weekly quests start counting</t>
+          <t xml:space="preserve">Doc is the first critter adopted</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 7 (from Nov 4)</t>
+          <t xml:space="preserve">Level 5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
@@ -427,22 +427,22 @@
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Win streak</t>
+          <t xml:space="preserve">Camp building + the mine</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Off until Nov 4, 2026, then shown as it happens: the flame counter under the hearts, a banner when free rocks fly, a line on the win card.</t>
+          <t xml:space="preserve">Camp callout on the first Home visit with build spots: the world glides to the campfire; tap a plus to build. Camp Lv 5 opens the ship.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game / Home</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">3 tiers: 1, 2, 3+ wins in a row = 1, 2, 3 free rocks thrown at the start of each level. A loss ends it unless a continue saves it; Restart ends it</t>
+          <t xml:space="preserve">The mine under the ship fills with materials over time</t>
         </is>
       </c>
     </row>
@@ -454,81 +454,81 @@
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Difficulty</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First Intermediate egg (3x3 hole)</t>
+          <t xml:space="preserve">Chest tray, Battle Pass, 7-Day Eggsperience</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">Home walkthrough: a free Common chest to unlock (gated taps), wins earn chests (3 wins each), the Battle Pass (hearts left become stars), the Eggsperience quests.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Level 7 deals two pieces; 8 all three, with a kinder deal</t>
+          <t xml:space="preserve">Stars, daily and weekly quests start counting</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 7+ (next Home visit)</t>
+          <t xml:space="preserve">Level 7 (from Nov 4)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Prompt</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Reminders ask</t>
+          <t xml:space="preserve">Win streak</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">"Stay in the loop?" card, then Android 13's permission prompt. Asked once; Settings &gt; Reminders toggles it.</t>
+          <t xml:space="preserve">Off until Nov 4, 2026, then shown as it happens: the flame counter under the hearts, a banner when free rocks fly, a line on the win card.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Game / Home</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Android only. Older Android needs no prompt</t>
+          <t xml:space="preserve">3 tiers: 1, 2, 3+ wins in a row = 1, 2, 3 free rocks thrown at the start of each level. A loss ends it unless a continue saves it; Restart ends it</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 8</t>
+          <t xml:space="preserve">Level 7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Booster</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Rocks (+2 free)</t>
+          <t xml:space="preserve">First Intermediate egg (3x3 hole)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card on the button: two rocks each land on a pair and finish the match.</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="0">
@@ -538,29 +538,29 @@
       </c>
       <c r="F14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Level 7 deals two pieces; 8 all three, with a kinder deal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 8</t>
+          <t xml:space="preserve">Level 7+ (next Home visit)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Sale</t>
+          <t xml:space="preserve">Prompt</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Starter Sprinkle</t>
+          <t xml:space="preserve">Reminders ask</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Pop-up on Home</t>
+          <t xml:space="preserve">"Stay in the loop?" card, then Android 13's permission prompt. Asked once; Settings &gt; Reminders toggles it.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
@@ -570,110 +570,110 @@
       </c>
       <c r="F15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Once ever</t>
+          <t xml:space="preserve">Android only. Older Android needs no prompt</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 10</t>
+          <t xml:space="preserve">Level 8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Feature</t>
+          <t xml:space="preserve">Booster</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Daily Egg + Daily Egg streak</t>
+          <t xml:space="preserve">Rocks (+2 free)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Callout on Home pointing at the Daily Egg tile.</t>
+          <t xml:space="preserve">Card on the button: two rocks each land on a pair and finish the match.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home / Daily Streaks</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Login streak is open from the start; the Daily Egg streak card unlocks here</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 10</t>
+          <t xml:space="preserve">Level 8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Blocker</t>
+          <t xml:space="preserve">Sale</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tie-downs (every other level from 10)</t>
+          <t xml:space="preserve">Starter Sprinkle</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2 cards: the camera turns to a tie-down; how it breaks; the counter by the hearts.</t>
+          <t xml:space="preserve">Pop-up on Home</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Once ever</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 12</t>
+          <t xml:space="preserve">Level 10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Prompt</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Rating ask</t>
+          <t xml:space="preserve">Daily Egg + Daily Egg streak</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">"Enjoying Egg Escape?" on Home after a win: Rate / Maybe later / No thanks.</t>
+          <t xml:space="preserve">Callout on Home pointing at the Daily Egg tile.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Home / Daily Streaks</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Android only. Again 25 levels later, 3 times at most; never after Rate or No thanks</t>
+          <t xml:space="preserve">Login streak is open from the start; the Daily Egg streak card unlocks here</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 13</t>
+          <t xml:space="preserve">Level 10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
@@ -683,12 +683,12 @@
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Geodes (odd levels from 13)</t>
+          <t xml:space="preserve">Tie-downs (every other level from 10)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: takes three hits, fires a rock when it cracks.</t>
+          <t xml:space="preserve">2 cards: the camera turns to a tie-down; how it breaks; the counter by the hearts.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
@@ -705,86 +705,86 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 15</t>
+          <t xml:space="preserve">Level 12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Difficulty</t>
+          <t xml:space="preserve">Prompt</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First Hard egg (4x4 hole)</t>
+          <t xml:space="preserve">Rating ask</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">"Enjoying Egg Escape?" on Home after a win: Rate / Maybe later / No thanks.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Android only. Again 25 levels later, 3 times at most; never after Rate or No thanks</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 15</t>
+          <t xml:space="preserve">Level 13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Sale</t>
+          <t xml:space="preserve">Blocker</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Flash Sale</t>
+          <t xml:space="preserve">Geodes (odd levels from 13)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Pop-up on Home</t>
+          <t xml:space="preserve">Card: takes three hits, fires a rock when it cracks.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Every 3 days from level 15</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">After level 17</t>
+          <t xml:space="preserve">Level 15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Challenge</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tutorial challenge (Intermediate egg, 3:00)</t>
+          <t xml:space="preserve">First Hard egg (4x4 hole)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2 cards: the clock; the rules (big coin bonus, buy a minute more, played once). The clock waits for them.</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
@@ -794,189 +794,189 @@
       </c>
       <c r="F22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Between 17 and 18. Played once; +3,000 coins on a win; time-out buy-out 1,000 coins = +1 min (+1 heart if one was lost)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 25</t>
+          <t xml:space="preserve">Level 15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Feature</t>
+          <t xml:space="preserve">Sale</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Clubs (teams) level gate</t>
+          <t xml:space="preserve">Flash Sale</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tab says "Teams open December 9!" until then</t>
+          <t xml:space="preserve">Pop-up on Home</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Bottom nav</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Needs level 25 AND Dec 9, 2026</t>
+          <t xml:space="preserve">Every 3 days from level 15</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 30</t>
+          <t xml:space="preserve">After level 17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Ads</t>
+          <t xml:space="preserve">Challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Interstitial ads</t>
+          <t xml:space="preserve">Tutorial challenge (Intermediate egg, 3:00)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">2 cards: the clock; the rules (big coin bonus, buy a minute more, played once). The clock waits for them.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">After wins</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Every 3rd win for non-payers; none for payers yet</t>
+          <t xml:space="preserve">Between 17 and 18. Played once; +3,000 coins on a win; time-out buy-out 1,000 coins = +1 min (+1 heart if one was lost)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 37</t>
+          <t xml:space="preserve">Level 25</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Difficulty</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First Extreme egg</t>
+          <t xml:space="preserve">Clubs (teams) level gate</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">PLAY turns deep red with an EXTREME tag; Home goes to its night scene</t>
+          <t xml:space="preserve">Tab says "Teams open December 9!" until then</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home / Game</t>
+          <t xml:space="preserve">Bottom nav</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Level 25 (planned Extreme) plays as Hard</t>
+          <t xml:space="preserve">Needs level 25 AND Dec 9, 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">After level 40</t>
+          <t xml:space="preserve">Level 30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Challenge</t>
+          <t xml:space="preserve">Ads</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First Extreme challenge (3:00)</t>
+          <t xml:space="preserve">Interstitial ads</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Same intro as the tutorial challenge if it is the player's first</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">After wins</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Then after 60, 80, 100... every 20 levels</t>
+          <t xml:space="preserve">Every 3rd win for non-payers; none for payers yet</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 50</t>
+          <t xml:space="preserve">Level 37</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Blocker</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Creeping vines (every 3rd level from 50)</t>
+          <t xml:space="preserve">First Extreme egg</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: a wrapped piece won't match or slide; pop next to it to cut it; vines spread.</t>
+          <t xml:space="preserve">PLAY turns deep red with an EXTREME tag; Home goes to its night scene</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Home / Game</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First vine level is a breather (Intermediate)</t>
+          <t xml:space="preserve">Level 25 (planned Extreme) plays as Hard</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 51</t>
+          <t xml:space="preserve">After level 40</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Difficulty</t>
+          <t xml:space="preserve">Challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Endless loop + slow ramp</t>
+          <t xml:space="preserve">First Extreme challenge (3:00)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">Same intro as the tutorial challenge if it is the player's first</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
@@ -986,61 +986,61 @@
       </c>
       <c r="F28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tiers repeat every 20 levels; one step harder every 50 levels up to level 551</t>
+          <t xml:space="preserve">Then after 60, 80, 100... every 20 levels</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 60</t>
+          <t xml:space="preserve">Level 50</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Ads</t>
+          <t xml:space="preserve">Blocker</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Interstitials every 2nd win</t>
+          <t xml:space="preserve">Creeping vines (every 3rd level from 50)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">Card: a wrapped piece won't match or slide; pop next to it to cut it; vines spread.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">After wins</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Non-payers; payers' first interstitials start here</t>
+          <t xml:space="preserve">First vine level is a breather (Intermediate)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 100</t>
+          <t xml:space="preserve">Level 51</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Blocker</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Padlocks &amp; key (every 3rd level from 100)</t>
+          <t xml:space="preserve">Endless loop + slow ramp</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2 cards: nothing breaks a locked stone; dig to the buried key.</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
@@ -1050,46 +1050,46 @@
       </c>
       <c r="F30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First lock level is a breather</t>
+          <t xml:space="preserve">Tiers repeat every 20 levels; one step harder every 50 levels up to level 551</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 150</t>
+          <t xml:space="preserve">Level 60</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Blocker</t>
+          <t xml:space="preserve">Ads</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Prism stones (every 3rd level from 150)</t>
+          <t xml:space="preserve">Interstitials every 2nd win</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: only a match of the prism's own colour next to it breaks it; the Any Piece counts as every colour.</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">After wins</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Rocks and bombs bounce off</t>
+          <t xml:space="preserve">Non-payers; payers' first interstitials start here</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 200</t>
+          <t xml:space="preserve">Level 100</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Fog (every 3rd level from 200)</t>
+          <t xml:space="preserve">Padlocks &amp; key (every 3rd level from 100)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: hides colours; pop next to it to clear part; a bomb or rock clears the whole cloud.</t>
+          <t xml:space="preserve">2 cards: nothing breaks a locked stone; dig to the buried key.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
@@ -1114,44 +1114,108 @@
       </c>
       <c r="F32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First fog level is a breather</t>
+          <t xml:space="preserve">First lock level is a breather</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Level 150</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Blocker</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Prism stones (every 3rd level from 150)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Card: only a match of the prism's own colour next to it breaks it; the Any Piece counts as every colour.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Game</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Rocks and bombs bounce off</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Level 200</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Blocker</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Fog (every 3rd level from 200)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Card: hides colours; pop next to it to clear part; a bomb or rock clears the whole cloud.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Game</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">First fog level is a breather</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Camp Lv 5</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr" s="0">
+      <c r="B35" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Feature</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr" s="0">
+      <c r="C35" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Ship repairs</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr" s="0">
+      <c r="D35" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Shown by the camp: Camp Lv 5 opens the ship's parts</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr" s="0">
+      <c r="E35" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr" s="0">
+      <c r="F35" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Not a level: from building the camp</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F33"/>
+  <autoFilter ref="A1:F35"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Piece counter: it reads "18 pieces left" ("1 piece left" on the last), and levels 1-5 are unlimited (TSLevels.UNLIMITED_PIECES_THROUGH: a budget of 0 -- no pill, no count, no "+5 pieces" on their lose card). One check, _has_piece_limit, now gates everything the counter does; its card shows on the first counted level with no other lesson (level 6 for a new player). Tests and the unlocks sheet updated.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/unlocks_and_tutorials.xlsx
+++ b/docs/unlocks_and_tutorials.xlsx
@@ -321,7 +321,7 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 1</t>
+          <t xml:space="preserve">Level 5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
@@ -331,22 +331,22 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Piece counter</t>
+          <t xml:space="preserve">Collection tab</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The pill under the tray counts down from the level's budget (no card yet)</t>
+          <t xml:space="preserve">Walkthrough after winning level 4: what the Collection is, a coin gift, tap Doc, tap Buy, Doc is yours; Collection levels add +1% materials.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Collection</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Each level's own budget (levels/piece_budgets.json), 10-31 pieces. Out of pieces: a heart buys one random piece; a continue or heart ad adds 5. Not on challenges</t>
+          <t xml:space="preserve">Doc is the first critter adopted</t>
         </is>
       </c>
     </row>
@@ -358,34 +358,34 @@
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Feature</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Piece counter card</t>
+          <t xml:space="preserve">Camp building + the mine</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">1 card on the counter: run out and each extra piece costs a heart, at random</t>
+          <t xml:space="preserve">Camp callout on the first Home visit with build spots: the world glides to the campfire; tap a plus to build. Camp Lv 5 opens the ship.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">Home</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The first level from 2 on with no other lesson (or the first time the pieces run out)</t>
+          <t xml:space="preserve">The mine under the ship fills with materials over time</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 5</t>
+          <t xml:space="preserve">Level 6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
@@ -395,54 +395,54 @@
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Collection tab</t>
+          <t xml:space="preserve">Piece counter</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Walkthrough after winning level 4: what the Collection is, a coin gift, tap Doc, tap Buy, Doc is yours; Collection levels add +1% materials.</t>
+          <t xml:space="preserve">The pill under the tray counts down: "18 pieces left" (levels 1-5 are unlimited)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Collection</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Doc is the first critter adopted</t>
+          <t xml:space="preserve">Each level's own budget (levels/piece_budgets.json), 10-31 pieces. Out of pieces: a heart buys one random piece; a continue or heart ad adds 5. Not on challenges</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 5</t>
+          <t xml:space="preserve">Level 6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Feature</t>
+          <t xml:space="preserve">Tutorial</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Camp building + the mine</t>
+          <t xml:space="preserve">Piece counter card</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Camp callout on the first Home visit with build spots: the world glides to the campfire; tap a plus to build. Camp Lv 5 opens the ship.</t>
+          <t xml:space="preserve">1 card on the counter: run out and each extra piece costs a heart, at random</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The mine under the ship fills with materials over time</t>
+          <t xml:space="preserve">The first counted level with no other lesson (or the first time the pieces run out)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Past level 50, a long win streak tightens the piece counter: a level started on a 5-win streak deals one piece fewer than its budget, on 7 or more two fewer (TSLevels.STREAK_CUT_AFTER, STREAK_CUTS, streak_piece_cut; applied in game.gd _start). Only levels that count toward the streak -- not the Daily Egg or challenges. Silent: the counter simply starts lower. Tests in tests/piece_counter_test; a row in the unlocks sheet.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/unlocks_and_tutorials.xlsx
+++ b/docs/unlocks_and_tutorials.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Dates and recurring" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By level'!$A$1:$F$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By level'!$A$1:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dates and recurring'!$A$1:$F$13</definedName>
   </definedNames>
 </workbook>
@@ -1057,71 +1057,71 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 60</t>
+          <t xml:space="preserve">Level 51+</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Ads</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Interstitials every 2nd win</t>
+          <t xml:space="preserve">Win-streak piece cut</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">None</t>
+          <t xml:space="preserve">None (silent)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">After wins</t>
+          <t xml:space="preserve">Game</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Non-payers; payers' first interstitials start here</t>
+          <t xml:space="preserve">On a 5-win streak a level deals 1 piece fewer than its budget; on 7+, 2 fewer. Not the Daily Egg or challenges</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 100</t>
+          <t xml:space="preserve">Level 60</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Blocker</t>
+          <t xml:space="preserve">Ads</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Padlocks &amp; key (every 3rd level from 100)</t>
+          <t xml:space="preserve">Interstitials every 2nd win</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2 cards: nothing breaks a locked stone; dig to the buried key.</t>
+          <t xml:space="preserve">None</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Game</t>
+          <t xml:space="preserve">After wins</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First lock level is a breather</t>
+          <t xml:space="preserve">Non-payers; payers' first interstitials start here</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 150</t>
+          <t xml:space="preserve">Level 100</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Prism stones (every 3rd level from 150)</t>
+          <t xml:space="preserve">Padlocks &amp; key (every 3rd level from 100)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: only a match of the prism's own colour next to it breaks it; the Any Piece counts as every colour.</t>
+          <t xml:space="preserve">2 cards: nothing breaks a locked stone; dig to the buried key.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
@@ -1146,14 +1146,14 @@
       </c>
       <c r="F33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Rocks and bombs bounce off</t>
+          <t xml:space="preserve">First lock level is a breather</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Level 200</t>
+          <t xml:space="preserve">Level 150</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Fog (every 3rd level from 200)</t>
+          <t xml:space="preserve">Prism stones (every 3rd level from 150)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Card: hides colours; pop next to it to clear part; a bomb or rock clears the whole cloud.</t>
+          <t xml:space="preserve">Card: only a match of the prism's own colour next to it breaks it; the Any Piece counts as every colour.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
@@ -1178,44 +1178,76 @@
       </c>
       <c r="F34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First fog level is a breather</t>
+          <t xml:space="preserve">Rocks and bombs bounce off</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Level 200</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Blocker</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Fog (every 3rd level from 200)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Card: hides colours; pop next to it to clear part; a bomb or rock clears the whole cloud.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Game</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">First fog level is a breather</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Camp Lv 5</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr" s="0">
+      <c r="B36" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Feature</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr" s="0">
+      <c r="C36" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Ship repairs</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr" s="0">
+      <c r="D36" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Shown by the camp: Camp Lv 5 opens the ship's parts</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr" s="0">
+      <c r="E36" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr" s="0">
+      <c r="F36" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Not a level: from building the camp</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F35"/>
+  <autoFilter ref="A1:F36"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Win-streak piece cut past level 50 goes further: 3 pieces off from a 9-win streak, 4 from 11 (TSLevels.STREAK_CUTS; still 1 from 5 and 2 from 7). Challenge levels run on a 2-minute clock (CHALLENGE_SECONDS 180 -> 120); the intro card reads it, the tests now follow the constant, and the 1.2 release notes and unlocks sheet say 2 minutes.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/unlocks_and_tutorials.xlsx
+++ b/docs/unlocks_and_tutorials.xlsx
@@ -843,7 +843,7 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tutorial challenge (Intermediate egg, 3:00)</t>
+          <t xml:space="preserve">Tutorial challenge (Intermediate egg, 2:00)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
@@ -971,7 +971,7 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">First Extreme challenge (3:00)</t>
+          <t xml:space="preserve">First Extreme challenge (2:00)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="F31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">On a 5-win streak a level deals 1 piece fewer than its budget; on 7+, 2 fewer. Not the Daily Egg or challenges</t>
+          <t xml:space="preserve">On a 5-win streak a level deals 1 piece fewer than its budget; 7: 2 fewer; 9: 3; 11+: 4. Not the Daily Egg or challenges</t>
         </is>
       </c>
     </row>

</xml_diff>